<commit_message>
Relevé GSC de départ (15/10) + redirections 301 des anciennes pages en 404
/politique, /arabe, /projets, rk-services, meridien, /sitemap.xml

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEO/PLAN-VISIBILITE-2026-2027.xlsx
+++ b/SEO/PLAN-VISIBILITE-2026-2027.xlsx
@@ -4975,15 +4975,37 @@
           <t>oct. 2026 (départ)</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>285</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>à compter</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="H5" s="7" t="inlineStr"/>
       <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Relevé du 15/10 : impressions ×3 depuis juillet, page 2. 1re requête : « rédacteur web senegal » (27). 4 pages en 404 redirigées.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">

</xml_diff>